<commit_message>
ng: update some forms
</commit_message>
<xml_diff>
--- a/ONCHO/Impact Assessments/Nigeria/2026/ng_oncho_stop_2605_1_site_stop_bn.xlsx
+++ b/ONCHO/Impact Assessments/Nigeria/2026/ng_oncho_stop_2605_1_site_stop_bn.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\ONCHO\Impact Assessments\Nigeria\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FB134BA-9803-4ED5-A234-C802B92BBB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C299E513-6A2E-473C-BBED-9EB99237C55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="237">
   <si>
     <t>type</t>
   </si>
@@ -392,12 +392,6 @@
     <t>${c_cluster_name}</t>
   </si>
   <si>
-    <t>ng_oncho_stop_2605_1_site_stop_bn</t>
-  </si>
-  <si>
-    <t>(Benue - 2026 May) - 1. Site Form</t>
-  </si>
-  <si>
     <t>BENUE</t>
   </si>
   <si>
@@ -407,9 +401,6 @@
     <t>APA</t>
   </si>
   <si>
-    <t>BUKURU</t>
-  </si>
-  <si>
     <t>BURUKU</t>
   </si>
   <si>
@@ -428,9 +419,6 @@
     <t>KATSINA-ALA</t>
   </si>
   <si>
-    <t>KONSHISA</t>
-  </si>
-  <si>
     <t>KWANDE</t>
   </si>
   <si>
@@ -449,9 +437,6 @@
     <t>OKPOKWU</t>
   </si>
   <si>
-    <t>OTURKPO</t>
-  </si>
-  <si>
     <t>UKUM</t>
   </si>
   <si>
@@ -464,39 +449,9 @@
     <t>IKPELE</t>
   </si>
   <si>
-    <t>OGBAI</t>
-  </si>
-  <si>
     <t>OWETO</t>
   </si>
   <si>
-    <t>OTURKPO - WETO ROAD</t>
-  </si>
-  <si>
-    <t>AJIO</t>
-  </si>
-  <si>
-    <t>AKOVOLWO</t>
-  </si>
-  <si>
-    <t>ANULE</t>
-  </si>
-  <si>
-    <t>BUTER</t>
-  </si>
-  <si>
-    <t>IHEMBA</t>
-  </si>
-  <si>
-    <t>METU</t>
-  </si>
-  <si>
-    <t>MINDE</t>
-  </si>
-  <si>
-    <t>SUSU</t>
-  </si>
-  <si>
     <t>DOGO</t>
   </si>
   <si>
@@ -512,36 +467,9 @@
     <t>JANGERIGERI</t>
   </si>
   <si>
-    <t>MBAGIR III</t>
-  </si>
-  <si>
-    <t>TYONDUN</t>
-  </si>
-  <si>
     <t>UDEI</t>
   </si>
   <si>
-    <t>YUSHEWE</t>
-  </si>
-  <si>
-    <t>YONOV</t>
-  </si>
-  <si>
-    <t>IBOR</t>
-  </si>
-  <si>
-    <t>UDUDU</t>
-  </si>
-  <si>
-    <t>MBAMTSAR</t>
-  </si>
-  <si>
-    <t>TOR DONGA</t>
-  </si>
-  <si>
-    <t>IKIRIYE ADUM</t>
-  </si>
-  <si>
     <t>AJIO-OBUDU ROAD</t>
   </si>
   <si>
@@ -566,190 +494,256 @@
     <t>USHAI</t>
   </si>
   <si>
-    <t>WAYA</t>
-  </si>
-  <si>
     <t>MBAYONGO LOGO 1</t>
   </si>
   <si>
-    <t>MBAKYONGU</t>
-  </si>
-  <si>
-    <t>IKINGO</t>
-  </si>
-  <si>
-    <t>OJEKWE</t>
-  </si>
-  <si>
-    <t>ICHAMA</t>
-  </si>
-  <si>
-    <t>UGBOKOLO</t>
-  </si>
-  <si>
-    <t>AKPACHI</t>
-  </si>
-  <si>
     <t>BEDE</t>
   </si>
   <si>
-    <t>TSE GYUBA</t>
-  </si>
-  <si>
     <t>AKPAGHER</t>
   </si>
   <si>
-    <t>TYOBAN</t>
-  </si>
-  <si>
     <t>. &gt; 1970 and . &lt;= 2026</t>
   </si>
   <si>
     <t>BEN_AGA_O_001</t>
   </si>
   <si>
-    <t>BEN_AGA_O_002</t>
-  </si>
-  <si>
-    <t>BEN_BUK_D_003</t>
-  </si>
-  <si>
-    <t>BEN_GBO_A_004</t>
-  </si>
-  <si>
-    <t>BEN_GUM_T_005</t>
-  </si>
-  <si>
-    <t>BEN_GUM_U_006</t>
-  </si>
-  <si>
-    <t>BEN_GUM_Y_007</t>
-  </si>
-  <si>
-    <t>BEN_GUM_M_008</t>
-  </si>
-  <si>
-    <t>BEN_GWE_Y_009</t>
-  </si>
-  <si>
-    <t>BEN_GWE_I_010</t>
-  </si>
-  <si>
-    <t>BEN_GWE_U_011</t>
-  </si>
-  <si>
-    <t>BEN_KAT_M_012</t>
-  </si>
-  <si>
-    <t>BEN_KAT_T_013</t>
-  </si>
-  <si>
-    <t>BEN_KWA_G_014</t>
-  </si>
-  <si>
-    <t>BEN_KWA_K_015</t>
-  </si>
-  <si>
-    <t>BEN_KWA_M_016</t>
-  </si>
-  <si>
-    <t>BEN_KWA_W_017</t>
-  </si>
-  <si>
-    <t>BEN_KON_I_018</t>
-  </si>
-  <si>
-    <t>BEN_OJU_O_019</t>
-  </si>
-  <si>
-    <t>BEN_OKP_I_020</t>
-  </si>
-  <si>
-    <t>BEN_OKP_U_021</t>
-  </si>
-  <si>
-    <t>BEN_OTU_A_022</t>
-  </si>
-  <si>
-    <t>BEN_UKU_B_023</t>
-  </si>
-  <si>
-    <t>BEN_UKU_T_024</t>
-  </si>
-  <si>
-    <t>BEN_USH_A_025</t>
-  </si>
-  <si>
-    <t>BEN_USH_T_026</t>
-  </si>
-  <si>
-    <t>BEN_BUR_U_027</t>
-  </si>
-  <si>
-    <t>BEN_MAK_M_028</t>
-  </si>
-  <si>
-    <t>BEN_LOG_M_029</t>
-  </si>
-  <si>
-    <t>BEN_OBI_I_030</t>
-  </si>
-  <si>
-    <t>BEN_AGA_A_031</t>
-  </si>
-  <si>
-    <t>BEN_AGA_I_032</t>
-  </si>
-  <si>
-    <t>BEN_APA_O_033</t>
-  </si>
-  <si>
-    <t>BEN_BEN_A_034</t>
-  </si>
-  <si>
-    <t>BEN_BEN_A_035</t>
-  </si>
-  <si>
-    <t>BEN_BEN_A_036</t>
-  </si>
-  <si>
-    <t>BEN_BEN_B_037</t>
-  </si>
-  <si>
-    <t>BEN_BEN_I_038</t>
-  </si>
-  <si>
-    <t>BEN_BEN_K_039</t>
-  </si>
-  <si>
-    <t>BEN_BEN_M_040</t>
-  </si>
-  <si>
-    <t>BEN_BEN_M_041</t>
-  </si>
-  <si>
-    <t>BEN_BEN_S_042</t>
-  </si>
-  <si>
-    <t>BEN_GUM_B_043</t>
-  </si>
-  <si>
-    <t>BEN_GUM_J_044</t>
-  </si>
-  <si>
-    <t>BEN_KWA_A_045</t>
-  </si>
-  <si>
-    <t>BEN_KWA_I_046</t>
-  </si>
-  <si>
-    <t>BEN_KWA_K_047</t>
-  </si>
-  <si>
-    <t>BEN_KWA_T_048</t>
-  </si>
-  <si>
-    <t>BEN_KWA_U_049</t>
+    <t>KONSHISHA</t>
+  </si>
+  <si>
+    <t>OTUKPO</t>
+  </si>
+  <si>
+    <t>OGBAI (IKPELE)</t>
+  </si>
+  <si>
+    <t>OTURKPO - WETO ROAD(OZANTELE)</t>
+  </si>
+  <si>
+    <t>GBAJIMBA IDP CAMP</t>
+  </si>
+  <si>
+    <t>IDP CAMP 1 DAUDU</t>
+  </si>
+  <si>
+    <t>IDP CAMP 2 DAUDU (UIKPAM)</t>
+  </si>
+  <si>
+    <t>IDP CAMP 3 DAUDU</t>
+  </si>
+  <si>
+    <t>TYOHEMBE</t>
+  </si>
+  <si>
+    <t>UNYIANDE</t>
+  </si>
+  <si>
+    <t>ANCHIHA</t>
+  </si>
+  <si>
+    <t>MBAAGIR</t>
+  </si>
+  <si>
+    <t>IDP CAMP NAKA</t>
+  </si>
+  <si>
+    <t>NAGI</t>
+  </si>
+  <si>
+    <t>NAKA</t>
+  </si>
+  <si>
+    <t>AMAAFU</t>
+  </si>
+  <si>
+    <t>JOO-MBATYOUGH</t>
+  </si>
+  <si>
+    <t>IKPEAKOR</t>
+  </si>
+  <si>
+    <t>REFUGEE SETTLEMENT (IKYOGEN)</t>
+  </si>
+  <si>
+    <t>IDP CAMP ANYIIN</t>
+  </si>
+  <si>
+    <t>MINDI</t>
+  </si>
+  <si>
+    <t>ADAKA</t>
+  </si>
+  <si>
+    <t>IDP CAMP ABAGANA</t>
+  </si>
+  <si>
+    <t>EKINGO</t>
+  </si>
+  <si>
+    <t>OJOKWE</t>
+  </si>
+  <si>
+    <t>ICHAMA CENTRAL</t>
+  </si>
+  <si>
+    <t>ODESSASSA I</t>
+  </si>
+  <si>
+    <t>AKPACHI UGBOJU</t>
+  </si>
+  <si>
+    <t>TSE GUBE</t>
+  </si>
+  <si>
+    <t>AKERIOR</t>
+  </si>
+  <si>
+    <t>BEN_AGA_A_002</t>
+  </si>
+  <si>
+    <t>BEN_AGA_I_003</t>
+  </si>
+  <si>
+    <t>BEN_AGA_O_004</t>
+  </si>
+  <si>
+    <t>BEN_APA_O_001</t>
+  </si>
+  <si>
+    <t>BEN_BUR_D_001</t>
+  </si>
+  <si>
+    <t>BEN_BUR_U_002</t>
+  </si>
+  <si>
+    <t>BEN_GBO_A_001</t>
+  </si>
+  <si>
+    <t>BEN_GUM_B_001</t>
+  </si>
+  <si>
+    <t>BEN_GUM_J_002</t>
+  </si>
+  <si>
+    <t>BEN_GUM_I_003</t>
+  </si>
+  <si>
+    <t>BEN_GUM_T_004</t>
+  </si>
+  <si>
+    <t>BEN_GUM_I_005</t>
+  </si>
+  <si>
+    <t>BEN_GUM_G_006</t>
+  </si>
+  <si>
+    <t>BEN_GUM_U_007</t>
+  </si>
+  <si>
+    <t>BEN_GUM_U_008</t>
+  </si>
+  <si>
+    <t>BEN_GUM_I_009</t>
+  </si>
+  <si>
+    <t>BEN_GWE_M_001</t>
+  </si>
+  <si>
+    <t>BEN_GWE_A_002</t>
+  </si>
+  <si>
+    <t>BEN_GWE_N_003</t>
+  </si>
+  <si>
+    <t>BEN_GWE_N_004</t>
+  </si>
+  <si>
+    <t>BEN_GWE_I_005</t>
+  </si>
+  <si>
+    <t>BEN_KAT_J_001</t>
+  </si>
+  <si>
+    <t>BEN_KAT_A_002</t>
+  </si>
+  <si>
+    <t>BEN_KON_I_001</t>
+  </si>
+  <si>
+    <t>BEN_KWA_G_001</t>
+  </si>
+  <si>
+    <t>BEN_KWA_K_002</t>
+  </si>
+  <si>
+    <t>BEN_KWA_A_003</t>
+  </si>
+  <si>
+    <t>BEN_KWA_A_004</t>
+  </si>
+  <si>
+    <t>BEN_KWA_I_005</t>
+  </si>
+  <si>
+    <t>BEN_KWA_K_006</t>
+  </si>
+  <si>
+    <t>BEN_KWA_T_007</t>
+  </si>
+  <si>
+    <t>BEN_KWA_U_008</t>
+  </si>
+  <si>
+    <t>BEN_KWA_R_009</t>
+  </si>
+  <si>
+    <t>BEN_LOG_M_001</t>
+  </si>
+  <si>
+    <t>BEN_LOG_M_002</t>
+  </si>
+  <si>
+    <t>BEN_LOG_I_003</t>
+  </si>
+  <si>
+    <t>BEN_MAK_I_001</t>
+  </si>
+  <si>
+    <t>BEN_MAK_A_002</t>
+  </si>
+  <si>
+    <t>BEN_OBI_E_001</t>
+  </si>
+  <si>
+    <t>BEN_OJU_O_001</t>
+  </si>
+  <si>
+    <t>BEN_OKP_O_001</t>
+  </si>
+  <si>
+    <t>BEN_OKP_I_002</t>
+  </si>
+  <si>
+    <t>BEN_OTU_A_001</t>
+  </si>
+  <si>
+    <t>BEN_UKU_B_001</t>
+  </si>
+  <si>
+    <t>BEN_UKU_T_002</t>
+  </si>
+  <si>
+    <t>BEN_USH_A_001</t>
+  </si>
+  <si>
+    <t>BEN_USH_M_002</t>
+  </si>
+  <si>
+    <t>(Benue - 2026 May) - 1. Site Form V2</t>
+  </si>
+  <si>
+    <t>ng_oncho_stop_2605_1_site_stop_bn_v2</t>
   </si>
 </sst>
 </file>
@@ -1617,7 +1611,7 @@
         <v>70</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>189</v>
+        <v>156</v>
       </c>
       <c r="G20" s="12" t="s">
         <v>71</v>
@@ -1681,7 +1675,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F144"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="16.375" customWidth="1"/>
@@ -1973,10 +1967,10 @@
         <v>84</v>
       </c>
       <c r="B23" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C23" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1984,13 +1978,13 @@
         <v>85</v>
       </c>
       <c r="B25" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C25" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1998,13 +1992,13 @@
         <v>85</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C26" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -2012,13 +2006,13 @@
         <v>85</v>
       </c>
       <c r="B27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -2026,13 +2020,13 @@
         <v>85</v>
       </c>
       <c r="B28" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C28" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2040,13 +2034,13 @@
         <v>85</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -2054,13 +2048,13 @@
         <v>85</v>
       </c>
       <c r="B30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -2068,13 +2062,13 @@
         <v>85</v>
       </c>
       <c r="B31" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C31" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2082,13 +2076,13 @@
         <v>85</v>
       </c>
       <c r="B32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -2096,13 +2090,13 @@
         <v>85</v>
       </c>
       <c r="B33" t="s">
-        <v>129</v>
+        <v>158</v>
       </c>
       <c r="C33" t="s">
-        <v>129</v>
+        <v>158</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -2110,13 +2104,13 @@
         <v>85</v>
       </c>
       <c r="B34" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C34" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -2124,13 +2118,13 @@
         <v>85</v>
       </c>
       <c r="B35" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C35" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -2138,13 +2132,13 @@
         <v>85</v>
       </c>
       <c r="B36" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C36" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -2152,13 +2146,13 @@
         <v>85</v>
       </c>
       <c r="B37" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C37" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D37" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -2166,13 +2160,13 @@
         <v>85</v>
       </c>
       <c r="B38" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C38" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D38" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -2180,13 +2174,13 @@
         <v>85</v>
       </c>
       <c r="B39" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C39" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D39" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -2194,13 +2188,13 @@
         <v>85</v>
       </c>
       <c r="B40" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="C40" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="D40" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -2208,13 +2202,13 @@
         <v>85</v>
       </c>
       <c r="B41" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C41" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D41" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -2222,58 +2216,58 @@
         <v>85</v>
       </c>
       <c r="B42" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C42" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D42" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" t="s">
-        <v>85</v>
-      </c>
-      <c r="B43" t="s">
-        <v>139</v>
-      </c>
-      <c r="C43" t="s">
-        <v>139</v>
-      </c>
-      <c r="D43" s="21" t="s">
-        <v>121</v>
-      </c>
+      <c r="D43" s="21"/>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B44" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C44" t="s">
-        <v>140</v>
-      </c>
-      <c r="D44" s="21" t="s">
-        <v>121</v>
+        <v>136</v>
+      </c>
+      <c r="E44" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="D45" s="21"/>
+      <c r="A45" t="s">
+        <v>86</v>
+      </c>
+      <c r="B45" t="s">
+        <v>137</v>
+      </c>
+      <c r="C45" t="s">
+        <v>137</v>
+      </c>
+      <c r="E45" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
         <v>86</v>
       </c>
       <c r="B46" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="C46" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="E46" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -2281,13 +2275,13 @@
         <v>86</v>
       </c>
       <c r="B47" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C47" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E47" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -2295,13 +2289,13 @@
         <v>86</v>
       </c>
       <c r="B48" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="C48" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="E48" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -2309,10 +2303,10 @@
         <v>86</v>
       </c>
       <c r="B49" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C49" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E49" t="s">
         <v>122</v>
@@ -2323,13 +2317,13 @@
         <v>86</v>
       </c>
       <c r="B50" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C50" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="E50" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -2337,13 +2331,13 @@
         <v>86</v>
       </c>
       <c r="B51" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="C51" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="E51" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -2351,13 +2345,13 @@
         <v>86</v>
       </c>
       <c r="B52" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C52" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E52" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -2365,13 +2359,13 @@
         <v>86</v>
       </c>
       <c r="B53" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C53" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="E53" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -2379,13 +2373,13 @@
         <v>86</v>
       </c>
       <c r="B54" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="C54" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="E54" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -2393,13 +2387,13 @@
         <v>86</v>
       </c>
       <c r="B55" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="C55" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="E55" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -2407,13 +2401,13 @@
         <v>86</v>
       </c>
       <c r="B56" t="s">
-        <v>132</v>
+        <v>165</v>
       </c>
       <c r="C56" t="s">
-        <v>132</v>
+        <v>165</v>
       </c>
       <c r="E56" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -2421,13 +2415,13 @@
         <v>86</v>
       </c>
       <c r="B57" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="C57" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="E57" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -2435,13 +2429,13 @@
         <v>86</v>
       </c>
       <c r="B58" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="C58" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="E58" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -2449,13 +2443,13 @@
         <v>86</v>
       </c>
       <c r="B59" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="C59" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="E59" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -2463,10 +2457,10 @@
         <v>86</v>
       </c>
       <c r="B60" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="C60" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="E60" t="s">
         <v>124</v>
@@ -2477,10 +2471,10 @@
         <v>86</v>
       </c>
       <c r="B61" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="C61" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="E61" t="s">
         <v>125</v>
@@ -2491,13 +2485,13 @@
         <v>86</v>
       </c>
       <c r="B62" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="C62" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="E62" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -2505,13 +2499,13 @@
         <v>86</v>
       </c>
       <c r="B63" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="C63" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="E63" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -2519,13 +2513,13 @@
         <v>86</v>
       </c>
       <c r="B64" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="C64" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="E64" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -2533,13 +2527,13 @@
         <v>86</v>
       </c>
       <c r="B65" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="C65" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="E65" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -2547,10 +2541,10 @@
         <v>86</v>
       </c>
       <c r="B66" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="C66" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="E66" t="s">
         <v>127</v>
@@ -2561,10 +2555,10 @@
         <v>86</v>
       </c>
       <c r="B67" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="C67" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="E67" t="s">
         <v>127</v>
@@ -2575,13 +2569,13 @@
         <v>86</v>
       </c>
       <c r="B68" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="C68" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="E68" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -2589,10 +2583,10 @@
         <v>86</v>
       </c>
       <c r="B69" t="s">
-        <v>163</v>
+        <v>141</v>
       </c>
       <c r="C69" t="s">
-        <v>163</v>
+        <v>141</v>
       </c>
       <c r="E69" t="s">
         <v>128</v>
@@ -2603,13 +2597,13 @@
         <v>86</v>
       </c>
       <c r="B70" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="C70" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="E70" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -2617,13 +2611,13 @@
         <v>86</v>
       </c>
       <c r="B71" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="C71" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="E71" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -2631,13 +2625,13 @@
         <v>86</v>
       </c>
       <c r="B72" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
       <c r="C72" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
       <c r="E72" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -2645,13 +2639,13 @@
         <v>86</v>
       </c>
       <c r="B73" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
       <c r="C73" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
       <c r="E73" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -2659,13 +2653,13 @@
         <v>86</v>
       </c>
       <c r="B74" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="C74" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="E74" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -2673,13 +2667,13 @@
         <v>86</v>
       </c>
       <c r="B75" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C75" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="E75" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -2687,13 +2681,13 @@
         <v>86</v>
       </c>
       <c r="B76" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C76" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="E76" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -2701,13 +2695,13 @@
         <v>86</v>
       </c>
       <c r="B77" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="C77" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="E77" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -2715,13 +2709,13 @@
         <v>86</v>
       </c>
       <c r="B78" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C78" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="E78" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -2729,13 +2723,13 @@
         <v>86</v>
       </c>
       <c r="B79" t="s">
-        <v>173</v>
+        <v>153</v>
       </c>
       <c r="C79" t="s">
-        <v>173</v>
+        <v>153</v>
       </c>
       <c r="E79" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -2743,13 +2737,13 @@
         <v>86</v>
       </c>
       <c r="B80" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C80" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="E80" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -2757,13 +2751,13 @@
         <v>86</v>
       </c>
       <c r="B81" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C81" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E81" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -2771,13 +2765,13 @@
         <v>86</v>
       </c>
       <c r="B82" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C82" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="E82" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -2785,13 +2779,13 @@
         <v>86</v>
       </c>
       <c r="B83" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C83" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E83" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -2799,13 +2793,13 @@
         <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C84" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E84" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -2813,13 +2807,13 @@
         <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C85" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="E85" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -2827,13 +2821,13 @@
         <v>86</v>
       </c>
       <c r="B86" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C86" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="E86" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -2841,13 +2835,13 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C87" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="E87" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -2855,13 +2849,13 @@
         <v>86</v>
       </c>
       <c r="B88" t="s">
-        <v>182</v>
+        <v>154</v>
       </c>
       <c r="C88" t="s">
-        <v>182</v>
+        <v>154</v>
       </c>
       <c r="E88" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -2869,13 +2863,13 @@
         <v>86</v>
       </c>
       <c r="B89" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C89" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E89" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -2883,13 +2877,13 @@
         <v>86</v>
       </c>
       <c r="B90" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C90" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E90" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -2897,46 +2891,32 @@
         <v>86</v>
       </c>
       <c r="B91" t="s">
-        <v>185</v>
+        <v>150</v>
       </c>
       <c r="C91" t="s">
-        <v>185</v>
+        <v>150</v>
       </c>
       <c r="E91" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6">
-      <c r="A92" t="s">
-        <v>86</v>
-      </c>
-      <c r="B92" t="s">
-        <v>186</v>
-      </c>
-      <c r="C92" t="s">
-        <v>186</v>
-      </c>
-      <c r="E92" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="A93" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="B93" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
       <c r="C93" t="s">
-        <v>187</v>
-      </c>
-      <c r="E93" t="s">
-        <v>140</v>
+        <v>157</v>
+      </c>
+      <c r="F93" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="94" spans="1:6">
       <c r="A94" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="B94" t="s">
         <v>188</v>
@@ -2944,8 +2924,22 @@
       <c r="C94" t="s">
         <v>188</v>
       </c>
-      <c r="E94" t="s">
-        <v>140</v>
+      <c r="F94" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
+      <c r="A95" t="s">
+        <v>108</v>
+      </c>
+      <c r="B95" t="s">
+        <v>189</v>
+      </c>
+      <c r="C95" t="s">
+        <v>189</v>
+      </c>
+      <c r="F95" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -2959,7 +2953,7 @@
         <v>190</v>
       </c>
       <c r="F96" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -2973,7 +2967,7 @@
         <v>191</v>
       </c>
       <c r="F97" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -2987,7 +2981,7 @@
         <v>192</v>
       </c>
       <c r="F98" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -3001,7 +2995,7 @@
         <v>193</v>
       </c>
       <c r="F99" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -3015,7 +3009,7 @@
         <v>194</v>
       </c>
       <c r="F100" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -3029,7 +3023,7 @@
         <v>195</v>
       </c>
       <c r="F101" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -3043,7 +3037,7 @@
         <v>196</v>
       </c>
       <c r="F102" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -3057,7 +3051,7 @@
         <v>197</v>
       </c>
       <c r="F103" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3071,7 +3065,7 @@
         <v>198</v>
       </c>
       <c r="F104" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3085,7 +3079,7 @@
         <v>199</v>
       </c>
       <c r="F105" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -3099,7 +3093,7 @@
         <v>200</v>
       </c>
       <c r="F106" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -3113,7 +3107,7 @@
         <v>201</v>
       </c>
       <c r="F107" t="s">
-        <v>166</v>
+        <v>144</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -3141,7 +3135,7 @@
         <v>203</v>
       </c>
       <c r="F109" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -3155,7 +3149,7 @@
         <v>204</v>
       </c>
       <c r="F110" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -3169,7 +3163,7 @@
         <v>205</v>
       </c>
       <c r="F111" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -3183,7 +3177,7 @@
         <v>206</v>
       </c>
       <c r="F112" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -3197,7 +3191,7 @@
         <v>207</v>
       </c>
       <c r="F113" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -3211,7 +3205,7 @@
         <v>208</v>
       </c>
       <c r="F114" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
     </row>
     <row r="115" spans="1:6">
@@ -3225,7 +3219,7 @@
         <v>209</v>
       </c>
       <c r="F115" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
     </row>
     <row r="116" spans="1:6">
@@ -3239,7 +3233,7 @@
         <v>210</v>
       </c>
       <c r="F116" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -3253,7 +3247,7 @@
         <v>211</v>
       </c>
       <c r="F117" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
     </row>
     <row r="118" spans="1:6">
@@ -3267,7 +3261,7 @@
         <v>212</v>
       </c>
       <c r="F118" t="s">
-        <v>185</v>
+        <v>146</v>
       </c>
     </row>
     <row r="119" spans="1:6">
@@ -3281,7 +3275,7 @@
         <v>213</v>
       </c>
       <c r="F119" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
     </row>
     <row r="120" spans="1:6">
@@ -3295,7 +3289,7 @@
         <v>214</v>
       </c>
       <c r="F120" t="s">
-        <v>187</v>
+        <v>141</v>
       </c>
     </row>
     <row r="121" spans="1:6">
@@ -3309,7 +3303,7 @@
         <v>215</v>
       </c>
       <c r="F121" t="s">
-        <v>188</v>
+        <v>145</v>
       </c>
     </row>
     <row r="122" spans="1:6">
@@ -3323,7 +3317,7 @@
         <v>216</v>
       </c>
       <c r="F122" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -3337,7 +3331,7 @@
         <v>217</v>
       </c>
       <c r="F123" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -3351,7 +3345,7 @@
         <v>218</v>
       </c>
       <c r="F124" t="s">
-        <v>178</v>
+        <v>151</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -3365,7 +3359,7 @@
         <v>219</v>
       </c>
       <c r="F125" t="s">
-        <v>180</v>
+        <v>152</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -3379,7 +3373,7 @@
         <v>220</v>
       </c>
       <c r="F126" t="s">
-        <v>141</v>
+        <v>176</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -3393,7 +3387,7 @@
         <v>221</v>
       </c>
       <c r="F127" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -3407,7 +3401,7 @@
         <v>222</v>
       </c>
       <c r="F128" t="s">
-        <v>145</v>
+        <v>178</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -3421,7 +3415,7 @@
         <v>223</v>
       </c>
       <c r="F129" t="s">
-        <v>146</v>
+        <v>177</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -3435,7 +3429,7 @@
         <v>224</v>
       </c>
       <c r="F130" t="s">
-        <v>147</v>
+        <v>180</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -3449,7 +3443,7 @@
         <v>225</v>
       </c>
       <c r="F131" t="s">
-        <v>148</v>
+        <v>179</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -3463,7 +3457,7 @@
         <v>226</v>
       </c>
       <c r="F132" t="s">
-        <v>149</v>
+        <v>181</v>
       </c>
     </row>
     <row r="133" spans="1:6">
@@ -3477,7 +3471,7 @@
         <v>227</v>
       </c>
       <c r="F133" t="s">
-        <v>150</v>
+        <v>182</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -3491,7 +3485,7 @@
         <v>228</v>
       </c>
       <c r="F134" t="s">
-        <v>132</v>
+        <v>184</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -3505,7 +3499,7 @@
         <v>229</v>
       </c>
       <c r="F135" t="s">
-        <v>151</v>
+        <v>183</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -3519,7 +3513,7 @@
         <v>230</v>
       </c>
       <c r="F136" t="s">
-        <v>152</v>
+        <v>185</v>
       </c>
     </row>
     <row r="137" spans="1:6">
@@ -3533,7 +3527,7 @@
         <v>231</v>
       </c>
       <c r="F137" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="138" spans="1:6">
@@ -3547,7 +3541,7 @@
         <v>232</v>
       </c>
       <c r="F138" t="s">
-        <v>157</v>
+        <v>186</v>
       </c>
     </row>
     <row r="139" spans="1:6">
@@ -3561,7 +3555,7 @@
         <v>233</v>
       </c>
       <c r="F139" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
     </row>
     <row r="140" spans="1:6">
@@ -3575,63 +3569,7 @@
         <v>234</v>
       </c>
       <c r="F140" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6">
-      <c r="A141" t="s">
-        <v>108</v>
-      </c>
-      <c r="B141" t="s">
-        <v>235</v>
-      </c>
-      <c r="C141" t="s">
-        <v>235</v>
-      </c>
-      <c r="F141" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6">
-      <c r="A142" t="s">
-        <v>108</v>
-      </c>
-      <c r="B142" t="s">
-        <v>236</v>
-      </c>
-      <c r="C142" t="s">
-        <v>236</v>
-      </c>
-      <c r="F142" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="143" spans="1:6">
-      <c r="A143" t="s">
-        <v>108</v>
-      </c>
-      <c r="B143" t="s">
-        <v>237</v>
-      </c>
-      <c r="C143" t="s">
-        <v>237</v>
-      </c>
-      <c r="F143" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6">
-      <c r="A144" t="s">
-        <v>108</v>
-      </c>
-      <c r="B144" t="s">
-        <v>238</v>
-      </c>
-      <c r="C144" t="s">
-        <v>238</v>
-      </c>
-      <c r="F144" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -3662,10 +3600,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="13" t="s">
-        <v>120</v>
+        <v>235</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>119</v>
+        <v>236</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>112</v>

</xml_diff>